<commit_message>
Contraste de precios ronda 5: soldadura, pinturas, seguridad y agregados
Verifica con evidencia de MercadoLibre VE y EPA Venezuela (USD):

- MT-ELECTRODO 4,80 → 5,00 USD/kg (6013: 4,50-9,14).
- MT-PINT-ANTICORR 7,20 → 8,00 USD/l (fondo anticorrosivo galón 30-52).
- MT-CERRADURA-MULTI 55 → 45 USD (multilock 25-95, mediana de seguridad).
- Confirma: MT-PINT-TRAFICO (9,2/l), MT-ARNES (55), MT-FLOTANTE (9,5),
  MT-ALAMBRE (1,9/kg), MT-GRAVILLA (24/m3).

Añade datos/contraste_mercado_2026-08d.json. Sin cambios de cobertura.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/descompuestos/05.04.01.030.xlsx
+++ b/basedatos_partidas/salida/descompuestos/05.04.01.030.xlsx
@@ -558,10 +558,10 @@
         <v>0.32</v>
       </c>
       <c r="G10" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="H10" t="n">
-        <v>1.54</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="11">
@@ -584,10 +584,10 @@
         <v>0.06</v>
       </c>
       <c r="G11" t="n">
-        <v>7.2</v>
+        <v>8</v>
       </c>
       <c r="H11" t="n">
-        <v>0.43</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="12">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1.97</v>
+        <v>2.08</v>
       </c>
     </row>
     <row r="13">
@@ -769,7 +769,7 @@
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>6.36</v>
+        <v>6.47</v>
       </c>
       <c r="H22" t="n">
         <v>0.06</v>
@@ -788,7 +788,7 @@
       </c>
       <c r="G23" s="4" t="n"/>
       <c r="H23" s="5" t="n">
-        <v>6.42</v>
+        <v>6.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>